<commit_message>
TICC-454 additional doc types
</commit_message>
<xml_diff>
--- a/work-in-progress/Peppol Code Lists - Document types v9.7.xlsx
+++ b/work-in-progress/Peppol Code Lists - Document types v9.7.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/philip/dev/git-peppol/edec-codelists/work-in-progress/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DBE495-88C1-6340-8ABD-B0E6C889A0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5AFE61-6A44-DE42-A483-007876BE5BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="899">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="896">
   <si>
     <t>urn:oasis:names:specification:ubl:schema:xsd:ApplicationResponse-2::ApplicationResponse##urn:www.cenbii.eu:transaction:biicoretrdm057:ver1.0:#urn:www.peppol.eu:bis:peppol1a:ver1.0::2.0</t>
   </si>
@@ -2217,20 +2217,6 @@
   </si>
   <si>
     <t>urn:un:unece:uncefact:data:standard:CrossIndustryInvoice:100::CrossIndustryInvoice##urn:cen.eu:en16931:2017#compliant#urn:peppol:france:billing:cius:1.0::D22B</t>
-  </si>
-  <si>
-    <t>cenbii-procid-ubl::urn:fdc:peppol.eu:2017:poacc:billing:01:1.0
-cenbii-procid-ubl::urn:peppol:france:billing:regulated
-cenbii-procid-ubl::urn:peppol:france:billing:non-regulated</t>
-  </si>
-  <si>
-    <t>cenbii-procid-ubl::urn:fdc:peppol.eu:2017:poacc:selfbilling:01:1.0
-cenbii-procid-ubl::urn:peppol:france:billing:regulated
-cenbii-procid-ubl::urn:peppol:france:billing:non-regulated</t>
-  </si>
-  <si>
-    <t>TICC-359
-TICC-365</t>
   </si>
   <si>
     <t>TICC-365</t>
@@ -3557,7 +3543,7 @@
         <v>343</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="G1" s="41" t="s">
         <v>393</v>
@@ -4109,7 +4095,7 @@
     </row>
     <row r="15" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="27" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="B15" s="27" t="s">
         <v>56</v>
@@ -4229,7 +4215,7 @@
     </row>
     <row r="18" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="B18" s="27" t="s">
         <v>56</v>
@@ -4429,7 +4415,7 @@
     </row>
     <row r="23" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A23" s="31" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="B23" s="27" t="s">
         <v>56</v>
@@ -4798,7 +4784,7 @@
         <v>345</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="I32" s="5" t="b">
         <v>0</v>
@@ -4817,12 +4803,12 @@
         <v>668</v>
       </c>
       <c r="N32" s="5" t="s">
-        <v>895</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>56</v>
@@ -4837,7 +4823,7 @@
         <v>345</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>710</v>
+        <v>895</v>
       </c>
       <c r="I33" s="5" t="b">
         <v>0</v>
@@ -4856,7 +4842,7 @@
         <v>669</v>
       </c>
       <c r="N33" s="5" t="s">
-        <v>707</v>
+        <v>892</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="48" x14ac:dyDescent="0.2">
@@ -5308,7 +5294,7 @@
     </row>
     <row r="45" spans="1:14" s="13" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A45" s="13" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>56</v>
@@ -5409,13 +5395,13 @@
         <v>470</v>
       </c>
       <c r="F47" s="15" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="G47" s="44">
         <v>46025</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="I47" s="13" t="b">
         <v>0</v>
@@ -5452,13 +5438,13 @@
         <v>470</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="G48" s="44">
         <v>46025</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="I48" s="13" t="b">
         <v>0</v>
@@ -5495,13 +5481,13 @@
         <v>344</v>
       </c>
       <c r="F49" s="33" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="G49" s="42">
         <v>46210</v>
       </c>
       <c r="H49" s="31" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="I49" s="31" t="b">
         <v>0</v>
@@ -5538,13 +5524,13 @@
         <v>344</v>
       </c>
       <c r="F50" s="33" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="G50" s="42">
         <v>46210</v>
       </c>
       <c r="H50" s="31" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="I50" s="31" t="b">
         <v>0</v>
@@ -5732,7 +5718,7 @@
         <v>345</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="I55" s="5" t="b">
         <v>0</v>
@@ -5751,7 +5737,7 @@
         <v>675</v>
       </c>
       <c r="N55" s="5" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
     </row>
     <row r="56" spans="1:14" ht="16" x14ac:dyDescent="0.2">
@@ -5969,7 +5955,7 @@
     </row>
     <row r="62" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>56</v>
@@ -6163,7 +6149,7 @@
     </row>
     <row r="67" spans="1:14" s="13" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A67" s="13" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>56</v>
@@ -6372,13 +6358,13 @@
         <v>470</v>
       </c>
       <c r="F72" s="17" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="G72" s="44">
         <v>46112</v>
       </c>
       <c r="H72" s="13" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="I72" s="13" t="b">
         <v>0</v>
@@ -6402,7 +6388,7 @@
     </row>
     <row r="73" spans="1:14" s="13" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A73" s="13" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="B73" s="14" t="s">
         <v>56</v>
@@ -6417,13 +6403,13 @@
         <v>470</v>
       </c>
       <c r="F73" s="17" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="G73" s="44">
         <v>46112</v>
       </c>
       <c r="H73" s="13" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="I73" s="13" t="b">
         <v>0</v>
@@ -6462,13 +6448,13 @@
         <v>470</v>
       </c>
       <c r="F74" s="17" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="G74" s="44">
         <v>46112</v>
       </c>
       <c r="H74" s="13" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="I74" s="13" t="b">
         <v>0</v>
@@ -6490,7 +6476,7 @@
     </row>
     <row r="75" spans="1:14" s="13" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A75" s="13" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="B75" s="14" t="s">
         <v>56</v>
@@ -6505,13 +6491,13 @@
         <v>470</v>
       </c>
       <c r="F75" s="17" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="G75" s="44">
         <v>46112</v>
       </c>
       <c r="H75" s="13" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="I75" s="13" t="b">
         <v>0</v>
@@ -6662,7 +6648,7 @@
     </row>
     <row r="79" spans="1:14" s="13" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A79" s="13" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="B79" s="14" t="s">
         <v>56</v>
@@ -6763,13 +6749,13 @@
         <v>344</v>
       </c>
       <c r="F81" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G81" s="45">
         <v>46235</v>
       </c>
       <c r="H81" s="31" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="I81" s="31" t="b">
         <v>0</v>
@@ -6791,7 +6777,7 @@
     </row>
     <row r="82" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A82" s="31" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="B82" s="27" t="s">
         <v>56</v>
@@ -6806,13 +6792,13 @@
         <v>344</v>
       </c>
       <c r="F82" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G82" s="45">
         <v>46235</v>
       </c>
       <c r="H82" s="31" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="I82" s="31" t="b">
         <v>0</v>
@@ -6892,13 +6878,13 @@
         <v>344</v>
       </c>
       <c r="F84" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G84" s="45">
         <v>46235</v>
       </c>
       <c r="H84" s="31" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="I84" s="31" t="b">
         <v>0</v>
@@ -6963,7 +6949,7 @@
     </row>
     <row r="86" spans="1:14" s="13" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A86" s="13" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="B86" s="14" t="s">
         <v>56</v>
@@ -7206,7 +7192,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="92" spans="1:14" s="31" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A92" s="31" t="s">
         <v>219</v>
       </c>
@@ -7285,7 +7271,7 @@
     </row>
     <row r="94" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>56</v>
@@ -7372,13 +7358,13 @@
         <v>344</v>
       </c>
       <c r="F96" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G96" s="42">
         <v>46235</v>
       </c>
       <c r="H96" s="31" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="I96" s="31" t="b">
         <v>0</v>
@@ -7400,7 +7386,7 @@
     </row>
     <row r="97" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A97" s="31" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="B97" s="27" t="s">
         <v>56</v>
@@ -7415,13 +7401,13 @@
         <v>344</v>
       </c>
       <c r="F97" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G97" s="42">
         <v>46235</v>
       </c>
       <c r="H97" s="31" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="I97" s="31" t="b">
         <v>0</v>
@@ -7501,13 +7487,13 @@
         <v>344</v>
       </c>
       <c r="F99" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G99" s="42">
         <v>46235</v>
       </c>
       <c r="H99" s="31" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="I99" s="31" t="b">
         <v>0</v>
@@ -7784,7 +7770,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="107" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A107" s="5" t="s">
         <v>176</v>
       </c>
@@ -9271,13 +9257,13 @@
         <v>344</v>
       </c>
       <c r="F148" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G148" s="42">
         <v>46235</v>
       </c>
       <c r="H148" s="31" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="I148" s="31" t="b">
         <v>0</v>
@@ -9298,7 +9284,7 @@
     </row>
     <row r="149" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A149" s="31" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="B149" s="27" t="s">
         <v>56</v>
@@ -9313,13 +9299,13 @@
         <v>344</v>
       </c>
       <c r="F149" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G149" s="42">
         <v>46235</v>
       </c>
       <c r="H149" s="31" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="I149" s="31" t="b">
         <v>0</v>
@@ -9355,13 +9341,13 @@
         <v>344</v>
       </c>
       <c r="F150" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G150" s="42">
         <v>46235</v>
       </c>
       <c r="H150" s="31" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="I150" s="31" t="b">
         <v>0</v>
@@ -9397,13 +9383,13 @@
         <v>344</v>
       </c>
       <c r="F151" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G151" s="42">
         <v>46235</v>
       </c>
       <c r="H151" s="31" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="I151" s="31" t="b">
         <v>0</v>
@@ -9424,7 +9410,7 @@
     </row>
     <row r="152" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A152" s="31" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="B152" s="27" t="s">
         <v>56</v>
@@ -9439,13 +9425,13 @@
         <v>344</v>
       </c>
       <c r="F152" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G152" s="42">
         <v>46235</v>
       </c>
       <c r="H152" s="31" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="I152" s="31" t="b">
         <v>0</v>
@@ -9481,13 +9467,13 @@
         <v>344</v>
       </c>
       <c r="F153" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G153" s="42">
         <v>46235</v>
       </c>
       <c r="H153" s="31" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="I153" s="31" t="b">
         <v>0</v>
@@ -10316,11 +10302,11 @@
         <v>344</v>
       </c>
       <c r="F175" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G175" s="42"/>
       <c r="H175" s="31" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="I175" s="31" t="b">
         <v>0</v>
@@ -10341,7 +10327,7 @@
     </row>
     <row r="176" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A176" s="31" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="B176" s="27" t="s">
         <v>56</v>
@@ -10356,11 +10342,11 @@
         <v>344</v>
       </c>
       <c r="F176" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G176" s="42"/>
       <c r="H176" s="31" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="I176" s="31" t="b">
         <v>0</v>
@@ -10396,11 +10382,11 @@
         <v>344</v>
       </c>
       <c r="F177" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G177" s="42"/>
       <c r="H177" s="31" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="I177" s="31" t="b">
         <v>0</v>
@@ -10436,11 +10422,11 @@
         <v>344</v>
       </c>
       <c r="F178" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G178" s="42"/>
       <c r="H178" s="31" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="I178" s="31" t="b">
         <v>0</v>
@@ -10461,7 +10447,7 @@
     </row>
     <row r="179" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A179" s="31" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="B179" s="27" t="s">
         <v>56</v>
@@ -10476,13 +10462,13 @@
         <v>344</v>
       </c>
       <c r="F179" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G179" s="42">
         <v>46235</v>
       </c>
       <c r="H179" s="31" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="I179" s="31" t="b">
         <v>0</v>
@@ -10518,11 +10504,11 @@
         <v>344</v>
       </c>
       <c r="F180" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G180" s="42"/>
       <c r="H180" s="31" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="I180" s="31" t="b">
         <v>0</v>
@@ -10627,7 +10613,7 @@
     </row>
     <row r="183" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A183" s="5" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="B183" s="4" t="s">
         <v>56</v>
@@ -10654,10 +10640,10 @@
         <v>1</v>
       </c>
       <c r="L183" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M183" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N183" s="37" t="s">
         <v>635</v>
@@ -10665,7 +10651,7 @@
     </row>
     <row r="184" spans="1:14" s="31" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A184" s="31" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
       <c r="B184" s="27" t="s">
         <v>56</v>
@@ -10680,11 +10666,11 @@
         <v>344</v>
       </c>
       <c r="F184" s="33" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G184" s="42"/>
       <c r="H184" s="31" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="I184" s="31" t="b">
         <v>0</v>
@@ -10696,10 +10682,10 @@
         <v>1</v>
       </c>
       <c r="L184" s="27" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M184" s="27" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N184" s="31" t="s">
         <v>421</v>
@@ -10707,7 +10693,7 @@
     </row>
     <row r="185" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A185" s="5" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="B185" s="4" t="s">
         <v>56</v>
@@ -10734,10 +10720,10 @@
         <v>1</v>
       </c>
       <c r="L185" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M185" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N185" s="12" t="s">
         <v>422</v>
@@ -10989,11 +10975,11 @@
         <v>344</v>
       </c>
       <c r="F192" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G192" s="42"/>
       <c r="H192" s="31" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
       <c r="I192" s="31" t="b">
         <v>0</v>
@@ -11014,7 +11000,7 @@
     </row>
     <row r="193" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A193" s="31" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="B193" s="27" t="s">
         <v>56</v>
@@ -11029,11 +11015,11 @@
         <v>344</v>
       </c>
       <c r="F193" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G193" s="42"/>
       <c r="H193" s="31" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
       <c r="I193" s="31" t="b">
         <v>0</v>
@@ -11069,11 +11055,11 @@
         <v>344</v>
       </c>
       <c r="F194" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G194" s="42"/>
       <c r="H194" s="31" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
       <c r="I194" s="31" t="b">
         <v>0</v>
@@ -11109,11 +11095,11 @@
         <v>344</v>
       </c>
       <c r="F195" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G195" s="42"/>
       <c r="H195" s="31" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="I195" s="31" t="b">
         <v>0</v>
@@ -11134,7 +11120,7 @@
     </row>
     <row r="196" spans="1:14" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A196" s="31" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="B196" s="27" t="s">
         <v>56</v>
@@ -11149,13 +11135,13 @@
         <v>344</v>
       </c>
       <c r="F196" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G196" s="42">
         <v>46235</v>
       </c>
       <c r="H196" s="31" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="I196" s="31" t="b">
         <v>0</v>
@@ -11191,11 +11177,11 @@
         <v>344</v>
       </c>
       <c r="F197" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G197" s="42"/>
       <c r="H197" s="31" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="I197" s="31" t="b">
         <v>0</v>
@@ -11835,7 +11821,7 @@
     </row>
     <row r="214" spans="1:14" s="13" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A214" s="38" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="B214" s="14" t="s">
         <v>56</v>
@@ -11850,13 +11836,13 @@
         <v>470</v>
       </c>
       <c r="F214" s="18" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="G214" s="44">
         <v>46025</v>
       </c>
       <c r="H214" s="13" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="I214" s="13" t="b">
         <v>0</v>
@@ -11868,10 +11854,10 @@
         <v>1</v>
       </c>
       <c r="L214" s="14" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M214" s="14" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N214" s="16" t="s">
         <v>539</v>
@@ -11879,7 +11865,7 @@
     </row>
     <row r="215" spans="1:14" s="13" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A215" s="38" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="B215" s="14" t="s">
         <v>56</v>
@@ -11894,13 +11880,13 @@
         <v>470</v>
       </c>
       <c r="F215" s="18" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="G215" s="44">
         <v>46025</v>
       </c>
       <c r="H215" s="13" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="I215" s="13" t="b">
         <v>0</v>
@@ -11912,10 +11898,10 @@
         <v>1</v>
       </c>
       <c r="L215" s="14" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M215" s="14" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N215" s="16" t="s">
         <v>540</v>
@@ -11923,7 +11909,7 @@
     </row>
     <row r="216" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A216" s="5" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="B216" s="4" t="s">
         <v>56</v>
@@ -11950,10 +11936,10 @@
         <v>1</v>
       </c>
       <c r="L216" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M216" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N216" s="36" t="s">
         <v>541</v>
@@ -11961,7 +11947,7 @@
     </row>
     <row r="217" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A217" s="5" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="B217" s="4" t="s">
         <v>56</v>
@@ -11976,7 +11962,7 @@
         <v>345</v>
       </c>
       <c r="H217" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
       <c r="I217" s="5" t="b">
         <v>0</v>
@@ -11988,18 +11974,18 @@
         <v>1</v>
       </c>
       <c r="L217" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M217" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N217" s="47" t="s">
-        <v>876</v>
+        <v>873</v>
       </c>
     </row>
     <row r="218" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A218" s="5" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="B218" s="4" t="s">
         <v>56</v>
@@ -12014,7 +12000,7 @@
         <v>345</v>
       </c>
       <c r="H218" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
       <c r="I218" s="5" t="b">
         <v>0</v>
@@ -12026,18 +12012,18 @@
         <v>1</v>
       </c>
       <c r="L218" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M218" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N218" s="47" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
     </row>
     <row r="219" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A219" s="5" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="B219" s="4" t="s">
         <v>56</v>
@@ -12064,10 +12050,10 @@
         <v>1</v>
       </c>
       <c r="L219" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M219" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N219" s="36" t="s">
         <v>542</v>
@@ -12218,7 +12204,7 @@
     </row>
     <row r="224" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A224" s="5" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="B224" s="5" t="s">
         <v>563</v>
@@ -12473,13 +12459,13 @@
         <v>470</v>
       </c>
       <c r="F230" s="39" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="G230" s="44">
         <v>45717</v>
       </c>
       <c r="H230" s="13" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="I230" s="13" t="b">
         <v>0</v>
@@ -12517,13 +12503,13 @@
         <v>470</v>
       </c>
       <c r="F231" s="39" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="G231" s="44">
         <v>45717</v>
       </c>
       <c r="H231" s="13" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="I231" s="13" t="b">
         <v>0</v>
@@ -12561,13 +12547,13 @@
         <v>470</v>
       </c>
       <c r="F232" s="39" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="G232" s="44">
         <v>45717</v>
       </c>
       <c r="H232" s="13" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="I232" s="13" t="b">
         <v>0</v>
@@ -12605,13 +12591,13 @@
         <v>470</v>
       </c>
       <c r="F233" s="39" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="G233" s="44">
         <v>45717</v>
       </c>
       <c r="H233" s="13" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="I233" s="13" t="b">
         <v>0</v>
@@ -12821,7 +12807,7 @@
     </row>
     <row r="239" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A239" s="5" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="B239" s="4" t="s">
         <v>56</v>
@@ -12926,7 +12912,7 @@
     </row>
     <row r="242" spans="1:14" s="31" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A242" s="31" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="B242" s="27" t="s">
         <v>56</v>
@@ -12941,13 +12927,13 @@
         <v>344</v>
       </c>
       <c r="F242" s="35" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G242" s="42">
         <v>46235</v>
       </c>
       <c r="H242" s="31" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="I242" s="31" t="b">
         <v>0</v>
@@ -13252,7 +13238,7 @@
         <v>45909</v>
       </c>
       <c r="H250" s="13" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="I250" s="13" t="b">
         <v>0</v>
@@ -13296,7 +13282,7 @@
         <v>45909</v>
       </c>
       <c r="H251" s="13" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="I251" s="13" t="b">
         <v>0</v>
@@ -13340,7 +13326,7 @@
         <v>45909</v>
       </c>
       <c r="H252" s="13" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="I252" s="13" t="b">
         <v>0</v>
@@ -13384,7 +13370,7 @@
         <v>45909</v>
       </c>
       <c r="H253" s="13" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="I253" s="13" t="b">
         <v>0</v>
@@ -13932,7 +13918,7 @@
     </row>
     <row r="269" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A269" s="5" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="B269" s="4" t="s">
         <v>56</v>
@@ -13947,7 +13933,7 @@
         <v>345</v>
       </c>
       <c r="H269" s="5" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="I269" s="5" t="b">
         <v>0</v>
@@ -13966,12 +13952,12 @@
         <v>668</v>
       </c>
       <c r="N269" s="5" t="s">
-        <v>896</v>
-      </c>
-    </row>
-    <row r="270" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="270" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A270" s="5" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="B270" s="4" t="s">
         <v>56</v>
@@ -13986,7 +13972,7 @@
         <v>345</v>
       </c>
       <c r="H270" s="5" t="s">
-        <v>709</v>
+        <v>894</v>
       </c>
       <c r="I270" s="5" t="b">
         <v>0</v>
@@ -14005,7 +13991,7 @@
         <v>669</v>
       </c>
       <c r="N270" s="5" t="s">
-        <v>708</v>
+        <v>893</v>
       </c>
     </row>
     <row r="271" spans="1:14" ht="32" x14ac:dyDescent="0.2">
@@ -14279,22 +14265,22 @@
     </row>
     <row r="278" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A278" s="5" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="B278" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C278" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="D278" s="24" t="s">
+        <v>712</v>
+      </c>
+      <c r="E278" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="H278" s="5" t="s">
         <v>713</v>
-      </c>
-      <c r="D278" s="24" t="s">
-        <v>715</v>
-      </c>
-      <c r="E278" s="20" t="s">
-        <v>345</v>
-      </c>
-      <c r="H278" s="5" t="s">
-        <v>716</v>
       </c>
       <c r="I278" s="5" t="b">
         <v>0</v>
@@ -14318,22 +14304,22 @@
     </row>
     <row r="279" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A279" s="5" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="B279" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C279" s="5" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="D279" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E279" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H279" s="5" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="I279" s="5" t="b">
         <v>0</v>
@@ -14357,22 +14343,22 @@
     </row>
     <row r="280" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="B280" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C280" s="1" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="D280" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E280" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H280" s="5" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="I280" s="5" t="b">
         <v>0</v>
@@ -14396,22 +14382,22 @@
     </row>
     <row r="281" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="B281" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C281" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="D281" s="24" t="s">
+        <v>712</v>
+      </c>
+      <c r="E281" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="H281" s="5" t="s">
         <v>722</v>
-      </c>
-      <c r="D281" s="24" t="s">
-        <v>715</v>
-      </c>
-      <c r="E281" s="20" t="s">
-        <v>345</v>
-      </c>
-      <c r="H281" s="5" t="s">
-        <v>725</v>
       </c>
       <c r="I281" s="5" t="b">
         <v>0</v>
@@ -14435,22 +14421,22 @@
     </row>
     <row r="282" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="B282" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="D282" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E282" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H282" s="5" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="I282" s="5" t="b">
         <v>0</v>
@@ -14474,22 +14460,22 @@
     </row>
     <row r="283" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="B283" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C283" s="1" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="D283" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E283" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H283" s="5" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="I283" s="5" t="b">
         <v>0</v>
@@ -14513,28 +14499,28 @@
     </row>
     <row r="284" spans="1:14" s="13" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A284" s="13" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="B284" s="13" t="s">
         <v>563</v>
       </c>
       <c r="C284" s="13" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="D284" s="25" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E284" s="21" t="s">
         <v>470</v>
       </c>
       <c r="F284" s="39" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G284" s="44">
         <v>46112</v>
       </c>
       <c r="H284" s="13" t="s">
-        <v>867</v>
+        <v>864</v>
       </c>
       <c r="I284" s="13" t="b">
         <v>0</v>
@@ -14548,36 +14534,36 @@
         <v>111</v>
       </c>
       <c r="M284" s="14" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="N284" s="13" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
     </row>
     <row r="285" spans="1:14" s="13" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A285" s="13" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="B285" s="13" t="s">
         <v>563</v>
       </c>
       <c r="C285" s="13" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="D285" s="25" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E285" s="21" t="s">
         <v>470</v>
       </c>
       <c r="F285" s="39" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="G285" s="44">
         <v>46112</v>
       </c>
       <c r="H285" s="13" t="s">
-        <v>867</v>
+        <v>864</v>
       </c>
       <c r="I285" s="13" t="b">
         <v>0</v>
@@ -14591,30 +14577,30 @@
         <v>111</v>
       </c>
       <c r="M285" s="14" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="N285" s="13" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
     </row>
     <row r="286" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A286" s="5" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="B286" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C286" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="D286" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E286" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H286" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I286" s="5" t="b">
         <v>0</v>
@@ -14624,33 +14610,33 @@
         <v>1</v>
       </c>
       <c r="L286" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M286" s="4" t="s">
         <v>668</v>
       </c>
       <c r="N286" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="287" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A287" s="5" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="B287" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C287" s="5" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="D287" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E287" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H287" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I287" s="5" t="b">
         <v>0</v>
@@ -14660,33 +14646,33 @@
         <v>1</v>
       </c>
       <c r="L287" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M287" s="4" t="s">
         <v>669</v>
       </c>
       <c r="N287" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="288" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A288" s="5" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="B288" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C288" s="5" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="D288" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E288" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H288" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I288" s="5" t="b">
         <v>0</v>
@@ -14696,33 +14682,33 @@
         <v>1</v>
       </c>
       <c r="L288" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M288" s="4" t="s">
         <v>667</v>
       </c>
       <c r="N288" s="5" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
     </row>
     <row r="289" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A289" s="5" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="B289" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C289" s="5" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="D289" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E289" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H289" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I289" s="5" t="b">
         <v>0</v>
@@ -14732,33 +14718,33 @@
         <v>1</v>
       </c>
       <c r="L289" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M289" s="4" t="s">
         <v>670</v>
       </c>
       <c r="N289" s="5" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
     </row>
     <row r="290" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A290" s="5" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="B290" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C290" s="5" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="D290" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E290" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H290" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I290" s="5" t="b">
         <v>0</v>
@@ -14768,33 +14754,33 @@
         <v>1</v>
       </c>
       <c r="L290" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M290" s="4" t="s">
         <v>671</v>
       </c>
       <c r="N290" s="5" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="291" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A291" s="5" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="B291" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C291" s="5" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="D291" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E291" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H291" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I291" s="5" t="b">
         <v>0</v>
@@ -14804,33 +14790,33 @@
         <v>1</v>
       </c>
       <c r="L291" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M291" s="4" t="s">
         <v>668</v>
       </c>
       <c r="N291" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="292" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A292" s="5" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="B292" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C292" s="5" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="D292" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E292" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H292" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I292" s="5" t="b">
         <v>0</v>
@@ -14840,33 +14826,33 @@
         <v>1</v>
       </c>
       <c r="L292" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M292" s="4" t="s">
         <v>667</v>
       </c>
       <c r="N292" s="5" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
     </row>
     <row r="293" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A293" s="5" t="s">
+        <v>769</v>
+      </c>
+      <c r="B293" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C293" s="5" t="s">
         <v>772</v>
       </c>
-      <c r="B293" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C293" s="5" t="s">
-        <v>775</v>
-      </c>
       <c r="D293" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E293" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H293" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I293" s="5" t="b">
         <v>0</v>
@@ -14876,33 +14862,33 @@
         <v>1</v>
       </c>
       <c r="L293" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M293" s="4" t="s">
         <v>670</v>
       </c>
       <c r="N293" s="5" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
     </row>
     <row r="294" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A294" s="5" t="s">
+        <v>770</v>
+      </c>
+      <c r="B294" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C294" s="5" t="s">
         <v>773</v>
       </c>
-      <c r="B294" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C294" s="5" t="s">
-        <v>776</v>
-      </c>
       <c r="D294" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E294" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H294" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I294" s="5" t="b">
         <v>0</v>
@@ -14912,33 +14898,33 @@
         <v>1</v>
       </c>
       <c r="L294" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M294" s="4" t="s">
         <v>671</v>
       </c>
       <c r="N294" s="5" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="295" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A295" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="B295" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C295" s="5" t="s">
         <v>774</v>
       </c>
-      <c r="B295" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C295" s="5" t="s">
-        <v>777</v>
-      </c>
       <c r="D295" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E295" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H295" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I295" s="5" t="b">
         <v>0</v>
@@ -14948,33 +14934,33 @@
         <v>1</v>
       </c>
       <c r="L295" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M295" s="4" t="s">
         <v>668</v>
       </c>
       <c r="N295" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="296" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A296" s="5" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="B296" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C296" s="5" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="D296" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E296" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H296" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I296" s="5" t="b">
         <v>0</v>
@@ -14984,33 +14970,33 @@
         <v>1</v>
       </c>
       <c r="L296" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M296" s="4" t="s">
         <v>667</v>
       </c>
       <c r="N296" s="5" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
     </row>
     <row r="297" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A297" s="5" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="B297" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C297" s="5" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D297" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E297" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H297" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I297" s="5" t="b">
         <v>0</v>
@@ -15020,33 +15006,33 @@
         <v>1</v>
       </c>
       <c r="L297" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M297" s="4" t="s">
         <v>668</v>
       </c>
       <c r="N297" s="5" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="298" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A298" s="5" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="B298" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C298" s="5" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="D298" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E298" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H298" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I298" s="5" t="b">
         <v>0</v>
@@ -15056,33 +15042,33 @@
         <v>1</v>
       </c>
       <c r="L298" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M298" s="4" t="s">
         <v>667</v>
       </c>
       <c r="N298" s="5" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
     </row>
     <row r="299" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A299" s="5" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="B299" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C299" s="5" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="D299" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E299" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H299" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I299" s="5" t="b">
         <v>0</v>
@@ -15092,33 +15078,33 @@
         <v>1</v>
       </c>
       <c r="L299" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M299" s="4" t="s">
         <v>670</v>
       </c>
       <c r="N299" s="5" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
     </row>
     <row r="300" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A300" s="5" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="B300" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C300" s="5" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="D300" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E300" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H300" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I300" s="5" t="b">
         <v>0</v>
@@ -15128,33 +15114,33 @@
         <v>1</v>
       </c>
       <c r="L300" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M300" s="4" t="s">
         <v>671</v>
       </c>
       <c r="N300" s="5" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="301" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A301" s="5" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="B301" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C301" s="5" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="D301" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E301" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H301" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I301" s="5" t="b">
         <v>0</v>
@@ -15164,33 +15150,33 @@
         <v>1</v>
       </c>
       <c r="L301" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M301" s="4" t="s">
         <v>668</v>
       </c>
       <c r="N301" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="302" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A302" s="5" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="B302" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C302" s="5" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="D302" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E302" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H302" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I302" s="5" t="b">
         <v>0</v>
@@ -15200,33 +15186,33 @@
         <v>1</v>
       </c>
       <c r="L302" s="4" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="M302" s="4" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="N302" s="5" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
     </row>
     <row r="303" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A303" s="5" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B303" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C303" s="5" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="D303" s="24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E303" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H303" s="5" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="I303" s="5" t="b">
         <v>0</v>
@@ -15246,22 +15232,22 @@
     </row>
     <row r="304" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A304" s="5" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="B304" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C304" s="5" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="D304" s="24" t="s">
+        <v>804</v>
+      </c>
+      <c r="E304" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="H304" s="5" t="s">
         <v>807</v>
-      </c>
-      <c r="E304" s="20" t="s">
-        <v>345</v>
-      </c>
-      <c r="H304" s="5" t="s">
-        <v>810</v>
       </c>
       <c r="I304" s="5" t="b">
         <v>0</v>
@@ -15274,30 +15260,30 @@
         <v>415</v>
       </c>
       <c r="M304" s="4" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="N304" s="5" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
     </row>
     <row r="305" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A305" s="5" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="B305" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C305" s="5" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="D305" s="24" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="E305" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H305" s="5" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="I305" s="5" t="b">
         <v>0</v>
@@ -15309,30 +15295,30 @@
         <v>555</v>
       </c>
       <c r="M305" s="4" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="N305" s="5" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
     </row>
     <row r="306" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="B306" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C306" s="1" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="D306" s="24" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="E306" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H306" s="5" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="I306" s="5" t="b">
         <v>0</v>
@@ -15356,22 +15342,22 @@
     </row>
     <row r="307" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="B307" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C307" s="1" t="s">
+        <v>818</v>
+      </c>
+      <c r="D307" s="24" t="s">
+        <v>820</v>
+      </c>
+      <c r="E307" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="H307" s="5" t="s">
         <v>821</v>
-      </c>
-      <c r="D307" s="24" t="s">
-        <v>823</v>
-      </c>
-      <c r="E307" s="20" t="s">
-        <v>345</v>
-      </c>
-      <c r="H307" s="5" t="s">
-        <v>824</v>
       </c>
       <c r="I307" s="5" t="b">
         <v>0</v>
@@ -15395,22 +15381,22 @@
     </row>
     <row r="308" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="B308" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C308" s="5" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="D308" s="24" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="E308" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H308" s="5" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="I308" s="5" t="b">
         <v>0</v>
@@ -15423,33 +15409,33 @@
         <v>1</v>
       </c>
       <c r="L308" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M308" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N308" s="5" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
     </row>
     <row r="309" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A309" s="5" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="B309" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C309" s="5" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="D309" s="24" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="E309" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H309" s="5" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="I309" s="5" t="b">
         <v>0</v>
@@ -15461,33 +15447,33 @@
         <v>1</v>
       </c>
       <c r="L309" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M309" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N309" s="47" t="s">
-        <v>873</v>
+        <v>870</v>
       </c>
     </row>
     <row r="310" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A310" s="5" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="B310" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C310" s="5" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="D310" s="24" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="E310" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H310" s="5" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="I310" s="5" t="b">
         <v>0</v>
@@ -15499,33 +15485,33 @@
         <v>1</v>
       </c>
       <c r="L310" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="M310" s="4" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="N310" s="47" t="s">
-        <v>874</v>
+        <v>871</v>
       </c>
     </row>
     <row r="311" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="B311" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C311" s="1" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="D311" s="24" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="E311" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H311" s="5" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="I311" s="5" t="b">
         <v>0</v>
@@ -15548,22 +15534,22 @@
     </row>
     <row r="312" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="B312" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C312" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="D312" s="24" t="s">
         <v>851</v>
       </c>
-      <c r="D312" s="24" t="s">
-        <v>854</v>
-      </c>
       <c r="E312" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H312" s="5" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="I312" s="5" t="b">
         <v>0</v>
@@ -15586,22 +15572,22 @@
     </row>
     <row r="313" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="B313" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C313" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="D313" s="24" t="s">
+        <v>851</v>
+      </c>
+      <c r="E313" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="H313" s="5" t="s">
         <v>852</v>
-      </c>
-      <c r="D313" s="24" t="s">
-        <v>854</v>
-      </c>
-      <c r="E313" s="20" t="s">
-        <v>345</v>
-      </c>
-      <c r="H313" s="5" t="s">
-        <v>855</v>
       </c>
       <c r="I313" s="5" t="b">
         <v>0</v>
@@ -15624,22 +15610,22 @@
     </row>
     <row r="314" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
       <c r="B314" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C314" s="1" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="D314" s="24" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="E314" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H314" s="5" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="I314" s="5" t="b">
         <v>0</v>
@@ -15662,23 +15648,23 @@
     </row>
     <row r="315" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="B315" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C315" s="1" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
       <c r="D315" s="24" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="E315" s="20" t="s">
         <v>345</v>
       </c>
       <c r="F315" s="46"/>
       <c r="H315" s="5" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="I315" s="5" t="b">
         <v>0</v>
@@ -15691,30 +15677,30 @@
         <v>111</v>
       </c>
       <c r="M315" s="4" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="N315" s="5" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
     </row>
     <row r="316" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
       <c r="B316" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C316" s="1" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="D316" s="24" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="E316" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H316" s="5" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="I316" s="5" t="b">
         <v>0</v>
@@ -15737,22 +15723,22 @@
     </row>
     <row r="317" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="B317" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C317" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="D317" s="24" t="s">
+        <v>876</v>
+      </c>
+      <c r="E317" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="H317" s="5" t="s">
         <v>886</v>
-      </c>
-      <c r="D317" s="24" t="s">
-        <v>879</v>
-      </c>
-      <c r="E317" s="20" t="s">
-        <v>345</v>
-      </c>
-      <c r="H317" s="5" t="s">
-        <v>889</v>
       </c>
       <c r="I317" s="5" t="b">
         <v>0</v>
@@ -15775,22 +15761,22 @@
     </row>
     <row r="318" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="B318" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C318" s="1" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="D318" s="24" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="E318" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H318" s="5" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="I318" s="5" t="b">
         <v>0</v>
@@ -15813,22 +15799,22 @@
     </row>
     <row r="319" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="B319" s="5" t="s">
         <v>563</v>
       </c>
       <c r="C319" s="1" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
       <c r="D319" s="24" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="E319" s="20" t="s">
         <v>345</v>
       </c>
       <c r="H319" s="5" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="I319" s="5" t="b">
         <v>0</v>
@@ -15851,23 +15837,23 @@
     </row>
     <row r="320" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="B320" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C320" s="1" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="D320" s="24" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="E320" s="20" t="s">
         <v>345</v>
       </c>
       <c r="F320" s="46"/>
       <c r="H320" s="5" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="I320" s="5" t="b">
         <v>0</v>
@@ -15880,31 +15866,31 @@
         <v>111</v>
       </c>
       <c r="M320" s="4" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="N320" s="5" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
     </row>
     <row r="321" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="B321" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C321" s="1" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="D321" s="24" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="E321" s="20" t="s">
         <v>345</v>
       </c>
       <c r="F321" s="46"/>
       <c r="H321" s="5" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="I321" s="5" t="b">
         <v>0</v>
@@ -15917,10 +15903,10 @@
         <v>111</v>
       </c>
       <c r="M321" s="4" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="N321" s="5" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
     </row>
   </sheetData>

</xml_diff>